<commit_message>
Restore Aug 2025 data vintage
</commit_message>
<xml_diff>
--- a/output/tables/results.xlsx
+++ b/output/tables/results.xlsx
@@ -413,19 +413,19 @@
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>1.84569148057862</v>
+        <v>1.85225038078164</v>
       </c>
       <c r="D2" t="n">
-        <v>1.05759165960529</v>
+        <v>1.05761302592482</v>
       </c>
       <c r="E2" t="n">
-        <v>0.994862981017951</v>
+        <v>0.997648146404922</v>
       </c>
       <c r="F2" t="n">
-        <v>1.23518459442348</v>
+        <v>1.23889759738603</v>
       </c>
       <c r="G2" t="n">
-        <v>0.386056637386733</v>
+        <v>0.386734463082823</v>
       </c>
     </row>
     <row r="3">
@@ -436,19 +436,19 @@
         <v>9</v>
       </c>
       <c r="C3" t="n">
-        <v>2.13997355298896</v>
+        <v>2.1554415688331</v>
       </c>
       <c r="D3" t="n">
-        <v>0.365400322166815</v>
+        <v>0.367939760726011</v>
       </c>
       <c r="E3" t="n">
-        <v>0.849223346116684</v>
+        <v>0.830277692475372</v>
       </c>
       <c r="F3" t="n">
-        <v>1.41110058869565</v>
+        <v>1.42660075684211</v>
       </c>
       <c r="G3" t="n">
-        <v>0.442245797561156</v>
+        <v>0.448694045499963</v>
       </c>
     </row>
     <row r="4">
@@ -459,19 +459,19 @@
         <v>10</v>
       </c>
       <c r="C4" t="n">
-        <v>2.03412576697783</v>
+        <v>1.99442830212796</v>
       </c>
       <c r="D4" t="n">
-        <v>0.590756011892373</v>
+        <v>0.560276650848672</v>
       </c>
       <c r="E4" t="n">
-        <v>0.695936350870835</v>
+        <v>0.568292950621204</v>
       </c>
       <c r="F4" t="n">
-        <v>1.35033791077539</v>
+        <v>1.36047563644861</v>
       </c>
       <c r="G4" t="n">
-        <v>0.421242240883273</v>
+        <v>0.429289597180518</v>
       </c>
     </row>
     <row r="5">
@@ -482,19 +482,19 @@
         <v>8</v>
       </c>
       <c r="C5" t="n">
-        <v>0.295070096629766</v>
+        <v>0.296265647866438</v>
       </c>
       <c r="D5" t="n">
-        <v>0.307100512780318</v>
+        <v>0.30708703762036</v>
       </c>
       <c r="E5" t="n">
-        <v>0.481752429381161</v>
+        <v>0.484298761973347</v>
       </c>
       <c r="F5" t="n">
-        <v>0.209947643176017</v>
+        <v>0.210249466974087</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0943436734702796</v>
+        <v>0.0948593338172351</v>
       </c>
     </row>
     <row r="6">
@@ -505,19 +505,19 @@
         <v>9</v>
       </c>
       <c r="C6" t="n">
-        <v>1.77166791867625</v>
+        <v>1.79724256992145</v>
       </c>
       <c r="D6" t="n">
-        <v>0.22852781007647</v>
+        <v>0.230857923375423</v>
       </c>
       <c r="E6" t="n">
-        <v>0.461648559853442</v>
+        <v>0.4901143806412</v>
       </c>
       <c r="F6" t="n">
-        <v>0.981141392173912</v>
+        <v>0.99829147368421</v>
       </c>
       <c r="G6" t="n">
-        <v>0.270941284918098</v>
+        <v>0.275750023923764</v>
       </c>
     </row>
     <row r="7">
@@ -528,19 +528,19 @@
         <v>10</v>
       </c>
       <c r="C7" t="n">
-        <v>1.52631892781384</v>
+        <v>1.53410494863442</v>
       </c>
       <c r="D7" t="n">
-        <v>0.357750046596848</v>
+        <v>0.364618156698427</v>
       </c>
       <c r="E7" t="n">
-        <v>0.347555209902929</v>
+        <v>0.365173281535133</v>
       </c>
       <c r="F7" t="n">
-        <v>0.803986502164758</v>
+        <v>0.791838118649366</v>
       </c>
       <c r="G7" t="n">
-        <v>0.20687846498454</v>
+        <v>0.201932451180729</v>
       </c>
     </row>
     <row r="8">
@@ -551,19 +551,19 @@
         <v>13</v>
       </c>
       <c r="C8" t="n">
-        <v>2.17096274788516</v>
+        <v>2.17882684265435</v>
       </c>
       <c r="D8" t="n">
-        <v>0.31326647294048</v>
+        <v>0.313232101183427</v>
       </c>
       <c r="E8" t="n">
-        <v>1.11548528444212</v>
+        <v>1.11267097879982</v>
       </c>
       <c r="F8" t="n">
-        <v>1.35236242750804</v>
+        <v>1.35732166230697</v>
       </c>
       <c r="G8" t="n">
-        <v>0.405599664504079</v>
+        <v>0.406652780790248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>